<commit_message>
style: uniformiser le format des références en attente de merge
Les références vers des profils FRCore non encore mergés sont maintenant
exprimées en commentaire inline sur la même ligne que la référence active.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com> a1dce5c1476e2dbca2511e99fc8b6e4f7212794a
</commit_message>
<xml_diff>
--- a/nr-doc-core-medication/ig/StructureDefinition-fr-core-medication-administration.xlsx
+++ b/nr-doc-core-medication/ig/StructureDefinition-fr-core-medication-administration.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-22T12:42:43+00:00</t>
+    <t>2026-06-22T14:38:01+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -581,7 +581,7 @@
 </t>
   </si>
   <si>
-    <t>Identifiant. L'entrée Traitement doit être identifiée de manière unique.</t>
+    <t>External identifier</t>
   </si>
   <si>
     <t>Identifiers associated with this Medication Administration that are defined by business processes and/or used to refer to it when a direct URL reference to the resource itself is not appropriate. They are business identifiers assigned to this resource by the performer or other systems and remain constant as the resource is updated and propagates from server to server.</t>

</xml_diff>

<commit_message>
Update FRCoreMedicationRequestProfile by removing fields
Removed intent and status cardinality from the profile. 90876b4ca7aa7dc65ed28372ed03e82e3ad85734
</commit_message>
<xml_diff>
--- a/nr-doc-core-medication/ig/StructureDefinition-fr-core-medication-administration.xlsx
+++ b/nr-doc-core-medication/ig/StructureDefinition-fr-core-medication-administration.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-29T12:42:10+00:00</t>
+    <t>2026-07-07T09:34:50+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1113,7 +1113,7 @@
     <t>extensible</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-human-substance-administration-site-cisis|20260420150249</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-human-substance-administration-site-cisis|20260619134041</t>
   </si>
   <si>
     <t>.approachSiteCode</t>

</xml_diff>

<commit_message>
Refine dosage.route binding description
Updated the binding description for dosage.route to remove versioning. 46a2e3350ccf3510345bf0d8c0529c32ca0816e9
</commit_message>
<xml_diff>
--- a/nr-doc-core-medication/ig/StructureDefinition-fr-core-medication-administration.xlsx
+++ b/nr-doc-core-medication/ig/StructureDefinition-fr-core-medication-administration.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-16T11:52:18+00:00</t>
+    <t>2026-07-16T13:43:45+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1131,7 +1131,7 @@
     <t>A code specifying the route or physiological path of administration of a therapeutic agent into or onto the patient.  For example, topical, intravenous, etc.</t>
   </si>
   <si>
-    <t>EDQM - Standard terms / classe ROA (0.4.0.127.0.16.1.1.2.1)</t>
+    <t>EDQM - Standard terms / classe ROA</t>
   </si>
   <si>
     <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-edqm|2.2.0</t>
@@ -5811,7 +5811,7 @@
         <v>80</v>
       </c>
       <c r="G37" t="s" s="2">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="H37" t="s" s="2">
         <v>79</v>

</xml_diff>